<commit_message>
W05 closeout: update Review123 template in 00_admin; archive W04 notebook
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/00_admin/AI_Capstone_Review123_Template.xlsx
+++ b/docs/00_admin/AI_Capstone_Review123_Template.xlsx
@@ -18,7 +18,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="69">
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t>Tên ĐATN</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+  </si>
   <si>
     <r>
       <rPr>
@@ -68,6 +88,104 @@
         <sz val="11.0"/>
         <u/>
       </rPr>
+      <t>Giảng viên Review</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve"> :</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t>Giảng viên Review</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t>Thời gian</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t>Thời gian</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <t>Tiêu chí</t>
+  </si>
+  <si>
+    <t>Gợi ý đánh giá/nhận xét</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Góp ý/nhận xét của GV Review</t>
+  </si>
+  <si>
+    <t>Những thay đổi sau lần Review2</t>
+  </si>
+  <si>
+    <t>Email các GV review</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
       <t>Mã ĐATN</t>
     </r>
     <r>
@@ -140,167 +258,122 @@
     </r>
   </si>
   <si>
-    <t>Tiêu chí</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Giảng viên Review</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <t>Gợi ý đánh giá/nhận xét</t>
-  </si>
-  <si>
-    <t>Góp ý/nhận xét của GV Review</t>
+    <t xml:space="preserve">Mục tiêu của đề tài (problem) </t>
+  </si>
+  <si>
+    <t>Phát biểu bài toán có đủ rõ ràng hay không ?</t>
   </si>
   <si>
     <t xml:space="preserve">Những thay đổi sau lần Review1 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Thời gian</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>:</t>
-    </r>
+    <t>Nguyễn Trọng Tài</t>
+  </si>
+  <si>
+    <t>taint51@fe.edu.vn</t>
   </si>
   <si>
     <t>Những thay đổi sau lần Review1 là gì ?
 Phản hồi sau lần review 1 từ nhóm ĐATN là gì ?</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Tên ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <t>Quản trị dự án/lập kế hoạch</t>
-  </si>
-  <si>
-    <t>Email các GV review</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Giảng viên Review</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> : </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Thời gian</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>:</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Mục tiêu của đề tài (problem) </t>
-  </si>
-  <si>
-    <t>Những thay đổi sau lần Review2</t>
-  </si>
-  <si>
-    <t>Lập kế hoạch có đầy đủ không ?</t>
+    <t>Kết quả cuối cùng là gi ? (proposed solution) 
+Kết quả mong muốn phải đạt được của đề tài là gì ?</t>
   </si>
   <si>
     <t>Những thay đổi sau lần Review2 là gì ?
 Phản hồi sau lần review 2 từ nhóm ĐATN là gì ?</t>
   </si>
   <si>
-    <t>Phát biểu bài toán có đủ rõ ràng hay không ?</t>
+    <t>Báo cáo khoa học/paper</t>
+  </si>
+  <si>
+    <t>Lê Phú Nguyên</t>
+  </si>
+  <si>
+    <t>nguyenlp9@fe.edu.vn</t>
+  </si>
+  <si>
+    <t>Software hoàn chỉnh</t>
+  </si>
+  <si>
+    <t>Nguyễn Quốc Trung</t>
+  </si>
+  <si>
+    <t>TrungNQ46@fe.edu.vn</t>
+  </si>
+  <si>
+    <t>Software prototype</t>
+  </si>
+  <si>
+    <t>Quản trị dự án/lập kế hoạch</t>
+  </si>
+  <si>
+    <t>Nguyễn Hồng Hải</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HaiNH51@fe.edu.vn </t>
+  </si>
+  <si>
+    <t>Framework/platform/library API</t>
+  </si>
+  <si>
+    <t>Vũ Hà Anh</t>
+  </si>
+  <si>
+    <t>Lập kế hoạch có đầy đủ không ?</t>
+  </si>
+  <si>
+    <t>AnhVH54@fe.edu.vn</t>
+  </si>
+  <si>
+    <t>Khác</t>
+  </si>
+  <si>
+    <t>Nguyễn Xuân Huy</t>
+  </si>
+  <si>
+    <t>huynx23@fe.edu.vn</t>
   </si>
   <si>
     <t>Phương pháp/mô hình quản trị dự án/công cụ hỗ trợ quản trị ?</t>
   </si>
   <si>
+    <t>Tính khả thi
+Xác định scope của đề tài</t>
+  </si>
+  <si>
     <t>Các phương pháp/hướng tiếp cận / mô hình giải quyết vấn đề đã đặt ra trong ĐATN</t>
   </si>
   <si>
-    <t>Nguyễn Trọng Tài</t>
-  </si>
-  <si>
-    <t>taint51@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Đánh giá kết quả của các phương pháp/hướng tiếp cận / mô hình giải đã đặt ra trong ĐATN</t>
+    <t>Dựa trên hướng tiếp cận nào; phương pháp/thuật toán/mô hình nào ==&gt; số lượng tìm hiểu là bao nhiêu ?</t>
+  </si>
+  <si>
+    <t>Dự kiến triển khai từ đầu hay tái sử dụng lại API/Framework/Platform có sẵn ?</t>
+  </si>
+  <si>
+    <t>Có cải tiến hay đưa ra mô hình, thuật toán mới không ? Số lượng là bao nhiêu ?</t>
+  </si>
+  <si>
+    <t>Tập dữ liệu mẫu tự xây dựng hay có sẵn ? Có thay đổi gì trên tập dữ liệu có sẵn hay không ?</t>
   </si>
   <si>
     <t>Hướng tiếp cận 1</t>
   </si>
   <si>
-    <t>Kết quả cuối cùng là gi ? (proposed solution) 
-Kết quả mong muốn phải đạt được của đề tài là gì ?</t>
+    <t>Giá trị của đề tài</t>
+  </si>
+  <si>
+    <t>Đề tài có tính thực tế không ? Có thể vận dụng được trong thực tế hay không ?</t>
   </si>
   <si>
     <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+  </si>
+  <si>
+    <t>Đề tài có ý nghĩa không (có giá trị, ý nghĩa khoa học hay không, nếu là báo cáo khoa học) ?</t>
+  </si>
+  <si>
+    <t>Đề tài có mới ?có  sáng tạo không ?</t>
   </si>
   <si>
     <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
@@ -308,94 +381,24 @@
 Thuật toán gì ? Thiết kế ra sao ?</t>
   </si>
   <si>
-    <t>Báo cáo khoa học/paper</t>
-  </si>
-  <si>
     <t>Huấn luyện / đánh giá mô hình như thế nào ?
 Độ phức tạp thuật toán như thế nào ?</t>
   </si>
   <si>
-    <t>Lê Phú Nguyên</t>
-  </si>
-  <si>
     <t>Tinh chỉnh các tham số như thế nào ?
 Cải tiến gì trong thuật toán ?</t>
   </si>
   <si>
-    <t>Khác</t>
+    <t>Đánh giá kết quả của các phương pháp/hướng tiếp cận / mô hình giải đã đặt ra trong ĐATN</t>
   </si>
   <si>
     <t>Hướng tiếp cận 2</t>
   </si>
   <si>
-    <t>nguyenlp9@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Software hoàn chỉnh</t>
-  </si>
-  <si>
-    <t>Nguyễn Quốc Trung</t>
-  </si>
-  <si>
-    <t>TrungNQ46@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Software prototype</t>
-  </si>
-  <si>
     <t>Hướng tiếp cận 3</t>
   </si>
   <si>
-    <t>Nguyễn Hồng Hải</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HaiNH51@fe.edu.vn </t>
-  </si>
-  <si>
-    <t>Framework/platform/library API</t>
-  </si>
-  <si>
-    <t>Vũ Hà Anh</t>
-  </si>
-  <si>
-    <t>AnhVH54@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Nguyễn Xuân Huy</t>
-  </si>
-  <si>
-    <t>huynx23@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Tính khả thi
-Xác định scope của đề tài</t>
-  </si>
-  <si>
-    <t>Dựa trên hướng tiếp cận nào; phương pháp/thuật toán/mô hình nào ==&gt; số lượng tìm hiểu là bao nhiêu ?</t>
-  </si>
-  <si>
-    <t>Dự kiến triển khai từ đầu hay tái sử dụng lại API/Framework/Platform có sẵn ?</t>
-  </si>
-  <si>
-    <t>Có cải tiến hay đưa ra mô hình, thuật toán mới không ? Số lượng là bao nhiêu ?</t>
-  </si>
-  <si>
-    <t>Tập dữ liệu mẫu tự xây dựng hay có sẵn ? Có thay đổi gì trên tập dữ liệu có sẵn hay không ?</t>
-  </si>
-  <si>
     <t>So sánh các phương pháp/ thảo luận / kết luận</t>
-  </si>
-  <si>
-    <t>Giá trị của đề tài</t>
-  </si>
-  <si>
-    <t>Đề tài có tính thực tế không ? Có thể vận dụng được trong thực tế hay không ?</t>
-  </si>
-  <si>
-    <t>Đề tài có ý nghĩa không (có giá trị, ý nghĩa khoa học hay không, nếu là báo cáo khoa học) ?</t>
-  </si>
-  <si>
-    <t>Đề tài có mới ?có  sáng tạo không ?</t>
   </si>
   <si>
     <r>
@@ -446,7 +449,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -463,6 +466,11 @@
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font/>
     <font>
@@ -532,6 +540,12 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -543,10 +557,12 @@
       </top>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
     </border>
     <border>
       <left style="thin">
@@ -590,14 +606,6 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-    </border>
-    <border>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -606,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -619,69 +627,72 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="9" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -917,168 +928,168 @@
   <sheetData>
     <row r="3">
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="8"/>
+        <v>10</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" ht="34.5" customHeight="1">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="14"/>
-      <c r="F8" s="8" t="s">
+      <c r="D8" s="10"/>
+      <c r="F8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" ht="34.5" customHeight="1">
+      <c r="B9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="D9" s="10"/>
+      <c r="F9" s="15" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" ht="34.5" customHeight="1">
-      <c r="B9" s="9" t="s">
+      <c r="G9" s="15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="34.5" customHeight="1">
+      <c r="B10" s="16"/>
+      <c r="C10" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="F10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="14"/>
-      <c r="F9" s="20" t="s">
+      <c r="G10" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" ht="34.5" customHeight="1">
+      <c r="B11" s="16"/>
+      <c r="C11" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="F11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="20" t="s">
+    </row>
+    <row r="12" ht="34.5" customHeight="1">
+      <c r="B12" s="16"/>
+      <c r="C12" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="F12" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" ht="34.5" customHeight="1">
-      <c r="B10" s="19"/>
-      <c r="C10" s="18" t="s">
+    <row r="13">
+      <c r="B13" s="20"/>
+      <c r="C13" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="F10" s="8" t="s">
+      <c r="D13" s="10"/>
+      <c r="F13" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G13" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" ht="34.5" customHeight="1">
-      <c r="B11" s="19"/>
-      <c r="C11" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="14"/>
-      <c r="F11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="8" t="s">
+    <row r="14" ht="34.5" customHeight="1">
+      <c r="B14" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="12" ht="34.5" customHeight="1">
-      <c r="B12" s="19"/>
-      <c r="C12" s="18" t="s">
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" ht="34.5" customHeight="1">
+      <c r="B15" s="16"/>
+      <c r="C15" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="14"/>
-      <c r="F12" s="21" t="s">
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" ht="34.5" customHeight="1">
+      <c r="B16" s="16"/>
+      <c r="C16" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" ht="34.5" customHeight="1">
+      <c r="B17" s="20"/>
+      <c r="C17" s="8" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="13"/>
-      <c r="C13" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="14"/>
-      <c r="F13" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="8" t="s">
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" ht="34.5" customHeight="1">
+      <c r="B18" s="12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="14" ht="34.5" customHeight="1">
-      <c r="B14" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15" ht="34.5" customHeight="1">
-      <c r="B15" s="19"/>
-      <c r="C15" s="12" t="s">
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" ht="34.5" customHeight="1">
+      <c r="B19" s="16"/>
+      <c r="C19" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16" ht="34.5" customHeight="1">
-      <c r="B16" s="19"/>
-      <c r="C16" s="12" t="s">
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" ht="34.5" customHeight="1">
+      <c r="B20" s="20"/>
+      <c r="C20" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="14"/>
-    </row>
-    <row r="17" ht="34.5" customHeight="1">
-      <c r="B17" s="13"/>
-      <c r="C17" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" ht="34.5" customHeight="1">
-      <c r="B18" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" ht="34.5" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" ht="34.5" customHeight="1">
-      <c r="B20" s="13"/>
-      <c r="C20" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="D20" s="10"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2093,179 +2104,184 @@
     <col customWidth="1" min="7" max="26" width="8.71"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="2">
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="1" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
-      <c r="B8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="6"/>
+      <c r="B8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" ht="31.5" customHeight="1">
-      <c r="B9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="6"/>
+      <c r="B9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="14"/>
     </row>
     <row r="10" ht="31.5" customHeight="1">
-      <c r="B10" s="13"/>
-      <c r="C10" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="6"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="14"/>
     </row>
     <row r="11" ht="31.5" customHeight="1">
-      <c r="B11" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="14"/>
+      <c r="B12" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="10"/>
     </row>
     <row r="13">
-      <c r="B13" s="19"/>
-      <c r="C13" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="14"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="10"/>
     </row>
     <row r="14">
-      <c r="B14" s="19"/>
-      <c r="C14" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="14"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="10"/>
     </row>
     <row r="15">
-      <c r="B15" s="19"/>
-      <c r="C15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="14"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="10"/>
     </row>
     <row r="16">
-      <c r="B16" s="13"/>
-      <c r="C16" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="14"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="10"/>
     </row>
     <row r="17" ht="48.75" customHeight="1">
-      <c r="B17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="14"/>
+      <c r="B17" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="10"/>
     </row>
     <row r="18" ht="48.75" customHeight="1">
-      <c r="B18" s="19"/>
-      <c r="C18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="14"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="10"/>
     </row>
     <row r="19" ht="48.75" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="14"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="10"/>
     </row>
     <row r="20" ht="48.75" customHeight="1">
-      <c r="B20" s="19"/>
-      <c r="C20" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="10"/>
     </row>
     <row r="21" ht="48.75" customHeight="1">
-      <c r="B21" s="13"/>
-      <c r="C21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="14"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="10"/>
     </row>
     <row r="22" ht="48.75" customHeight="1">
-      <c r="B22" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="14"/>
+      <c r="B22" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="10"/>
     </row>
     <row r="23" ht="48.75" customHeight="1">
-      <c r="B23" s="19"/>
-      <c r="C23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="14"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="10"/>
     </row>
     <row r="24" ht="48.75" customHeight="1">
-      <c r="B24" s="19"/>
-      <c r="C24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="14"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" s="10"/>
     </row>
     <row r="25" ht="48.75" customHeight="1">
-      <c r="B25" s="19"/>
-      <c r="C25" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="14"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="10"/>
     </row>
     <row r="26" ht="48.75" customHeight="1">
-      <c r="B26" s="13"/>
-      <c r="C26" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="14"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="10"/>
     </row>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>
@@ -3278,250 +3294,250 @@
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="6"/>
+      <c r="B8" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" ht="31.5" hidden="1" customHeight="1">
-      <c r="B9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>20</v>
+      <c r="B9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>37</v>
       </c>
       <c r="D9" s="3"/>
     </row>
     <row r="10" ht="31.5" hidden="1" customHeight="1">
-      <c r="B10" s="13"/>
-      <c r="C10" s="11" t="s">
-        <v>23</v>
+      <c r="B10" s="20"/>
+      <c r="C10" s="18" t="s">
+        <v>42</v>
       </c>
       <c r="D10" s="3"/>
     </row>
     <row r="11" ht="31.5" customHeight="1">
-      <c r="B11" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" ht="48.75" customHeight="1">
-      <c r="B12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="14"/>
+      <c r="B12" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="10"/>
     </row>
     <row r="13" ht="48.75" customHeight="1">
-      <c r="B13" s="19"/>
-      <c r="C13" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="14"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="10"/>
     </row>
     <row r="14" ht="48.75" customHeight="1">
-      <c r="B14" s="19"/>
-      <c r="C14" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="14"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="10"/>
     </row>
     <row r="15" ht="48.75" customHeight="1">
-      <c r="B15" s="19"/>
-      <c r="C15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="14"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="10"/>
     </row>
     <row r="16" ht="48.75" customHeight="1">
-      <c r="B16" s="13"/>
-      <c r="C16" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="14"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="10"/>
     </row>
     <row r="17" ht="48.75" customHeight="1">
-      <c r="B17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="14"/>
+      <c r="B17" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="10"/>
     </row>
     <row r="18" ht="48.75" customHeight="1">
-      <c r="B18" s="19"/>
-      <c r="C18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="14"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="10"/>
     </row>
     <row r="19" ht="48.75" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="14"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="10"/>
     </row>
     <row r="20" ht="48.75" customHeight="1">
-      <c r="B20" s="19"/>
-      <c r="C20" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="10"/>
     </row>
     <row r="21" ht="48.75" customHeight="1">
-      <c r="B21" s="13"/>
-      <c r="C21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="14"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="10"/>
     </row>
     <row r="22" ht="48.75" customHeight="1">
-      <c r="B22" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="14"/>
+      <c r="B22" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="10"/>
     </row>
     <row r="23" ht="48.75" customHeight="1">
-      <c r="B23" s="19"/>
-      <c r="C23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="14"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="10"/>
     </row>
     <row r="24" ht="48.75" customHeight="1">
-      <c r="B24" s="19"/>
-      <c r="C24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="14"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" s="10"/>
     </row>
     <row r="25" ht="48.75" customHeight="1">
-      <c r="B25" s="19"/>
-      <c r="C25" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="14"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="10"/>
     </row>
     <row r="26" ht="48.75" customHeight="1">
-      <c r="B26" s="13"/>
-      <c r="C26" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="14"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="10"/>
     </row>
     <row r="27" ht="33.75" customHeight="1">
-      <c r="B27" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
+      <c r="B27" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
     </row>
     <row r="28">
-      <c r="B28" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
+      <c r="B28" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
     </row>
     <row r="29" ht="30.0" customHeight="1">
-      <c r="B29" s="26" t="s">
-        <v>62</v>
+      <c r="B29" s="27" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
-      <c r="V30" s="27"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
+      <c r="V30" s="28"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
+      <c r="Z30" s="28"/>
     </row>
     <row r="31" ht="32.25" customHeight="1">
-      <c r="B31" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="31"/>
+      <c r="B31" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="32"/>
     </row>
     <row r="32" ht="32.25" customHeight="1">
-      <c r="B32" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="31"/>
+      <c r="B32" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="32"/>
     </row>
     <row r="33" ht="32.25" customHeight="1">
-      <c r="B33" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="31"/>
+      <c r="B33" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="32"/>
     </row>
     <row r="34" ht="32.25" customHeight="1">
-      <c r="B34" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="31"/>
+      <c r="B34" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="32"/>
     </row>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>

</xml_diff>